<commit_message>
Publish current working project state
</commit_message>
<xml_diff>
--- a/docs/exports/scraping-inventory.xlsx
+++ b/docs/exports/scraping-inventory.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scraping Inventory'!$A$1:$X$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scraping Inventory'!$A$1:$AC$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X45"/>
+  <dimension ref="A1:AC45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -491,20 +491,25 @@
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
-    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+    <col width="8" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="40" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,75 +560,100 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Live URLs Discovered</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Live Listings Parsed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Live Photos Downloaded</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Latest Live Run (UTC)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Live Product Buckets</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Fixture Listings Scraped</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Discovery Fixtures</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Discovery URLs Found</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Blocked/Error Fixtures</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Photos Scraped</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Has Description</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Has Geo (lat/lon)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Has Address/City</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Has Area (sqm)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Has Rooms</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Has Price</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Intents Covered</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Property Types Seen</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Connector Status</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -672,54 +702,73 @@
         <v>18000</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:32:08.324143+00:00</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Scaffold + discovery</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Core agency network with strong local branches.</t>
         </is>
@@ -768,54 +817,73 @@
         <v>35000</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:32:05.492715+00:00</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr">
+      <c r="AA3" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W3" s="2" t="inlineStr">
+      <c r="AB3" s="2" t="inlineStr">
         <is>
           <t>Scaffold + discovery</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>Strong coastal inventory, especially land and new-build.</t>
         </is>
@@ -864,54 +932,73 @@
         <v>12000</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1</v>
+        <v>249</v>
       </c>
       <c r="L4" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:42:37.971917+00:00</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr">
-        <is>
-          <t>Scaffold + discovery</t>
-        </is>
-      </c>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>Scaffold + discovery + live batch</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
         <is>
           <t>Important for new-build and foreign buyer inventory.</t>
         </is>
@@ -960,54 +1047,73 @@
         <v>120000</v>
       </c>
       <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09T09:41:11.623753+00:00</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="P5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="Q5" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="R5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="S5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="2" t="n">
+      <c r="T5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="R5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="2" t="n">
+      <c r="W5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U5" s="2" t="inlineStr">
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="V5" s="2" t="inlineStr">
+      <c r="AA5" s="2" t="inlineStr">
         <is>
           <t>apartment, house</t>
         </is>
       </c>
-      <c r="W5" s="2" t="inlineStr">
+      <c r="AB5" s="2" t="inlineStr">
         <is>
           <t>Full connector + discovery</t>
         </is>
       </c>
-      <c r="X5" s="2" t="inlineStr">
+      <c r="AC5" s="2" t="inlineStr">
         <is>
           <t>Crawl-friendly and broad national coverage.</t>
         </is>
@@ -1056,54 +1162,73 @@
         <v>200000</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1</v>
+        <v>254</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="L6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:30:52.841147+00:00</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U6" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr">
+      <c r="AA6" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W6" s="2" t="inlineStr">
-        <is>
-          <t>Scaffold + discovery</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="inlineStr">
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>Scaffold + discovery + live batch</t>
+        </is>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
         <is>
           <t>High-volume benchmark supply source.</t>
         </is>
@@ -1152,7 +1277,7 @@
         <v>90000</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
@@ -1160,46 +1285,61 @@
       <c r="L7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>1</v>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U7" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="AA7" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="AB7" s="2" t="inlineStr">
         <is>
           <t>Scaffold (headless needed)</t>
         </is>
       </c>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="AC7" s="2" t="inlineStr">
         <is>
           <t>403 and anti-bot patterns raise risk.</t>
         </is>
@@ -1248,54 +1388,73 @@
         <v>4000</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:32:16.250052+00:00</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
+      <c r="AA8" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W8" s="2" t="inlineStr">
+      <c r="AB8" s="2" t="inlineStr">
         <is>
           <t>Scaffold + discovery</t>
         </is>
       </c>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="AC8" s="2" t="inlineStr">
         <is>
           <t>Luxury coastal segment.</t>
         </is>
@@ -1344,54 +1503,73 @@
         <v>45000</v>
       </c>
       <c r="J9" s="2" t="n">
+        <v>257</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>1365</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T17:31:38.962595+00:00</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="P9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="Q9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" s="2" t="n">
+      <c r="R9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="2" t="n">
+      <c r="T9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="Q9" s="2" t="n">
+      <c r="V9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="R9" s="2" t="n">
+      <c r="W9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="S9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U9" s="2" t="inlineStr">
+      <c r="X9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr">
+      <c r="AA9" s="2" t="inlineStr">
         <is>
           <t>apartment, land</t>
         </is>
       </c>
-      <c r="W9" s="2" t="inlineStr">
-        <is>
-          <t>Full connector (API) + discovery</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>Full connector (API) + discovery + live batch</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
         <is>
           <t>Primary API-first classifieds source.</t>
         </is>
@@ -1440,54 +1618,69 @@
         <v>10000</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr">
+      <c r="AA10" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W10" s="2" t="inlineStr">
+      <c r="AB10" s="2" t="inlineStr">
         <is>
           <t>Scaffold + discovery</t>
         </is>
       </c>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="AC10" s="2" t="inlineStr">
         <is>
           <t>Cross-check source for foreign-buyer inventory.</t>
         </is>
@@ -1536,54 +1729,73 @@
         <v>15000</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:32:14.138810+00:00</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="R11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U11" s="2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr">
+      <c r="AA11" s="2" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W11" s="2" t="inlineStr">
+      <c r="AB11" s="2" t="inlineStr">
         <is>
           <t>Scaffold + discovery</t>
         </is>
       </c>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="AC11" s="2" t="inlineStr">
         <is>
           <t>High-value coastal and resort inventory.</t>
         </is>
@@ -1640,11 +1852,11 @@
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="3" t="n">
-        <v>0</v>
+      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O12" s="3" t="n">
         <v>0</v>
@@ -1664,22 +1876,37 @@
       <c r="T12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W12" s="3" t="inlineStr">
+      <c r="U12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB12" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X12" s="3" t="inlineStr">
+      <c r="AC12" s="3" t="inlineStr">
         <is>
           <t>Managed resort inventory.</t>
         </is>
@@ -1728,54 +1955,73 @@
         <v>8000</v>
       </c>
       <c r="J13" s="3" t="n">
+        <v>272</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>2487</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-08T16:54:12.900549+00:00</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="3" t="n">
+      <c r="P13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="O13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="3" t="n">
+      <c r="T13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="Q13" s="3" t="n">
+      <c r="V13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="R13" s="3" t="n">
+      <c r="W13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="S13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="3" t="n">
+      <c r="X13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="U13" s="3" t="inlineStr">
+      <c r="Z13" s="3" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V13" s="3" t="inlineStr">
+      <c r="AA13" s="3" t="inlineStr">
         <is>
           <t>apartment, land</t>
         </is>
       </c>
-      <c r="W13" s="3" t="inlineStr">
-        <is>
-          <t>Tier-2 stub connector</t>
-        </is>
-      </c>
-      <c r="X13" s="3" t="inlineStr">
+      <c r="AB13" s="3" t="inlineStr">
+        <is>
+          <t>Tier-2 stub connector + live batch</t>
+        </is>
+      </c>
+      <c r="AC13" s="3" t="inlineStr">
         <is>
           <t>Secondary but useful classifieds source.</t>
         </is>
@@ -1824,54 +2070,69 @@
         <v>22000</v>
       </c>
       <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="3" t="n">
+      <c r="P14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="3" t="n">
+      <c r="T14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="Q14" s="3" t="n">
+      <c r="V14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="R14" s="3" t="n">
+      <c r="W14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="S14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="3" t="n">
+      <c r="X14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="U14" s="3" t="inlineStr">
+      <c r="Z14" s="3" t="inlineStr">
         <is>
           <t>sale, short_term_rent</t>
         </is>
       </c>
-      <c r="V14" s="3" t="inlineStr">
+      <c r="AA14" s="3" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W14" s="3" t="inlineStr">
+      <c r="AB14" s="3" t="inlineStr">
         <is>
           <t>Tier-2 stub connector</t>
         </is>
       </c>
-      <c r="X14" s="3" t="inlineStr">
+      <c r="AC14" s="3" t="inlineStr">
         <is>
           <t>Needs cross-language dedupe.</t>
         </is>
@@ -1928,11 +2189,11 @@
       <c r="L15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="3" t="n">
-        <v>0</v>
+      <c r="M15" s="3" t="inlineStr"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O15" s="3" t="n">
         <v>0</v>
@@ -1952,22 +2213,37 @@
       <c r="T15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W15" s="3" t="inlineStr">
+      <c r="U15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB15" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X15" s="3" t="inlineStr">
+      <c r="AC15" s="3" t="inlineStr">
         <is>
           <t>Strong Varna-side project inventory.</t>
         </is>
@@ -2016,54 +2292,69 @@
         <v>6000</v>
       </c>
       <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="3" t="n">
+      <c r="P16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="O16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="3" t="n">
+      <c r="T16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="Q16" s="3" t="n">
+      <c r="V16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="R16" s="3" t="n">
+      <c r="W16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="S16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="3" t="n">
+      <c r="X16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="U16" s="3" t="inlineStr">
+      <c r="Z16" s="3" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V16" s="3" t="inlineStr">
+      <c r="AA16" s="3" t="inlineStr">
         <is>
           <t>house, project</t>
         </is>
       </c>
-      <c r="W16" s="3" t="inlineStr">
+      <c r="AB16" s="3" t="inlineStr">
         <is>
           <t>Tier-2 stub connector</t>
         </is>
       </c>
-      <c r="X16" s="3" t="inlineStr">
+      <c r="AC16" s="3" t="inlineStr">
         <is>
           <t>Important for Varna and project inventory.</t>
         </is>
@@ -2120,11 +2411,11 @@
       <c r="L17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="3" t="n">
-        <v>0</v>
+      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O17" s="3" t="n">
         <v>0</v>
@@ -2144,22 +2435,37 @@
       <c r="T17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U17" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V17" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W17" s="3" t="inlineStr">
+      <c r="U17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB17" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X17" s="3" t="inlineStr">
+      <c r="AC17" s="3" t="inlineStr">
         <is>
           <t>JS-heavy source with higher content-use risk.</t>
         </is>
@@ -2216,11 +2522,11 @@
       <c r="L18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="3" t="n">
-        <v>0</v>
+      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O18" s="3" t="n">
         <v>0</v>
@@ -2240,22 +2546,37 @@
       <c r="T18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W18" s="3" t="inlineStr">
+      <c r="U18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB18" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X18" s="3" t="inlineStr">
+      <c r="AC18" s="3" t="inlineStr">
         <is>
           <t>Terms indicate commercial data use requires authorization/payment.</t>
         </is>
@@ -2312,11 +2633,11 @@
       <c r="L19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>0</v>
+      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O19" s="3" t="n">
         <v>0</v>
@@ -2336,22 +2657,37 @@
       <c r="T19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U19" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V19" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W19" s="3" t="inlineStr">
+      <c r="U19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB19" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X19" s="3" t="inlineStr">
+      <c r="AC19" s="3" t="inlineStr">
         <is>
           <t>Secondary index for coastal supply.</t>
         </is>
@@ -2408,11 +2744,11 @@
       <c r="L20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>0</v>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O20" s="3" t="n">
         <v>0</v>
@@ -2432,22 +2768,37 @@
       <c r="T20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W20" s="3" t="inlineStr">
+      <c r="U20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB20" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X20" s="3" t="inlineStr">
+      <c r="AC20" s="3" t="inlineStr">
         <is>
           <t>Useful Varna-side agency inventory.</t>
         </is>
@@ -2504,11 +2855,11 @@
       <c r="L21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>0</v>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O21" s="3" t="n">
         <v>0</v>
@@ -2528,22 +2879,37 @@
       <c r="T21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W21" s="3" t="inlineStr">
+      <c r="U21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB21" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X21" s="3" t="inlineStr">
+      <c r="AC21" s="3" t="inlineStr">
         <is>
           <t>Hospitality intelligence more than core sale inventory.</t>
         </is>
@@ -2600,11 +2966,11 @@
       <c r="L22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="3" t="n">
-        <v>0</v>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O22" s="3" t="n">
         <v>0</v>
@@ -2624,22 +2990,37 @@
       <c r="T22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W22" s="3" t="inlineStr">
+      <c r="U22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB22" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X22" s="3" t="inlineStr">
+      <c r="AC22" s="3" t="inlineStr">
         <is>
           <t>Foreign-facing Alo network layer.</t>
         </is>
@@ -2696,11 +3077,11 @@
       <c r="L23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="3" t="n">
-        <v>0</v>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O23" s="3" t="n">
         <v>0</v>
@@ -2720,22 +3101,37 @@
       <c r="T23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W23" s="3" t="inlineStr">
+      <c r="U23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB23" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X23" s="3" t="inlineStr">
+      <c r="AC23" s="3" t="inlineStr">
         <is>
           <t>Map-driven browsing suggests structured geo data.</t>
         </is>
@@ -2792,11 +3188,11 @@
       <c r="L24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="3" t="n">
-        <v>0</v>
+      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O24" s="3" t="n">
         <v>0</v>
@@ -2816,22 +3212,37 @@
       <c r="T24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W24" s="3" t="inlineStr">
+      <c r="U24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB24" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X24" s="3" t="inlineStr">
+      <c r="AC24" s="3" t="inlineStr">
         <is>
           <t>Varna rental specialist.</t>
         </is>
@@ -2888,11 +3299,11 @@
       <c r="L25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="3" t="n">
-        <v>0</v>
+      <c r="M25" s="3" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O25" s="3" t="n">
         <v>0</v>
@@ -2912,22 +3323,37 @@
       <c r="T25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W25" s="3" t="inlineStr">
+      <c r="U25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB25" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X25" s="3" t="inlineStr">
+      <c r="AC25" s="3" t="inlineStr">
         <is>
           <t>Useful for worker and student rentals.</t>
         </is>
@@ -2984,11 +3410,11 @@
       <c r="L26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="3" t="n">
-        <v>0</v>
+      <c r="M26" s="3" t="inlineStr"/>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O26" s="3" t="n">
         <v>0</v>
@@ -3008,22 +3434,37 @@
       <c r="T26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W26" s="3" t="inlineStr">
+      <c r="U26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB26" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X26" s="3" t="inlineStr">
+      <c r="AC26" s="3" t="inlineStr">
         <is>
           <t>Luxury sea-segment pages.</t>
         </is>
@@ -3080,11 +3521,11 @@
       <c r="L27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="M27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="3" t="n">
-        <v>0</v>
+      <c r="M27" s="3" t="inlineStr"/>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O27" s="3" t="n">
         <v>0</v>
@@ -3104,22 +3545,37 @@
       <c r="T27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="U27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W27" s="3" t="inlineStr">
+      <c r="U27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB27" s="3" t="inlineStr">
         <is>
           <t>Not yet implemented</t>
         </is>
       </c>
-      <c r="X27" s="3" t="inlineStr">
+      <c r="AC27" s="3" t="inlineStr">
         <is>
           <t>Villa and guest-house coverage.</t>
         </is>
@@ -3168,54 +3624,73 @@
         <v>9000</v>
       </c>
       <c r="J28" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>249</v>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-08T17:18:17.189285+00:00</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="3" t="n">
+      <c r="P28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="O28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="3" t="n">
+      <c r="T28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="Q28" s="3" t="n">
+      <c r="V28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="R28" s="3" t="n">
+      <c r="W28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="S28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="3" t="n">
+      <c r="X28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="U28" s="3" t="inlineStr">
+      <c r="Z28" s="3" t="inlineStr">
         <is>
           <t>long_term_rent, sale</t>
         </is>
       </c>
-      <c r="V28" s="3" t="inlineStr">
+      <c r="AA28" s="3" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W28" s="3" t="inlineStr">
-        <is>
-          <t>Tier-2 stub connector</t>
-        </is>
-      </c>
-      <c r="X28" s="3" t="inlineStr">
+      <c r="AB28" s="3" t="inlineStr">
+        <is>
+          <t>Tier-2 stub connector + live batch</t>
+        </is>
+      </c>
+      <c r="AC28" s="3" t="inlineStr">
         <is>
           <t>Established agency with branch-driven supply.</t>
         </is>
@@ -3274,11 +3749,11 @@
       <c r="L29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="4" t="n">
-        <v>0</v>
+      <c r="M29" s="4" t="inlineStr"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O29" s="4" t="n">
         <v>0</v>
@@ -3298,22 +3773,37 @@
       <c r="T29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W29" s="4" t="inlineStr">
+      <c r="U29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA29" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X29" s="4" t="inlineStr">
+      <c r="AC29" s="4" t="inlineStr">
         <is>
           <t>Do not rely on scraping as a core acquisition path.</t>
         </is>
@@ -3372,11 +3862,11 @@
       <c r="L30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="4" t="n">
-        <v>0</v>
+      <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O30" s="4" t="n">
         <v>0</v>
@@ -3396,22 +3886,37 @@
       <c r="T30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V30" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W30" s="4" t="inlineStr">
+      <c r="U30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA30" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X30" s="4" t="inlineStr">
+      <c r="AC30" s="4" t="inlineStr">
         <is>
           <t>Use for coastal STR benchmarks.</t>
         </is>
@@ -3470,11 +3975,11 @@
       <c r="L31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="4" t="n">
-        <v>0</v>
+      <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O31" s="4" t="n">
         <v>0</v>
@@ -3494,22 +3999,37 @@
       <c r="T31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W31" s="4" t="inlineStr">
+      <c r="U31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA31" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB31" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X31" s="4" t="inlineStr">
+      <c r="AC31" s="4" t="inlineStr">
         <is>
           <t>Use for STR enrichment, not primary listings.</t>
         </is>
@@ -3558,54 +4078,69 @@
         <v>1224</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="inlineStr"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="M32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="4" t="n">
+      <c r="R32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="O32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S32" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="T32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U32" s="4" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="U32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
         <is>
           <t>auction_sale</t>
         </is>
       </c>
-      <c r="V32" s="4" t="inlineStr">
+      <c r="AA32" s="4" t="inlineStr">
         <is>
           <t>Къща</t>
         </is>
       </c>
-      <c r="W32" s="4" t="inlineStr">
+      <c r="AB32" s="4" t="inlineStr">
         <is>
           <t>Tier-3 stub (auction parser)</t>
         </is>
       </c>
-      <c r="X32" s="4" t="inlineStr">
+      <c r="AC32" s="4" t="inlineStr">
         <is>
           <t>Useful opportunistic inventory source.</t>
         </is>
@@ -3664,11 +4199,11 @@
       <c r="L33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="4" t="n">
-        <v>0</v>
+      <c r="M33" s="4" t="inlineStr"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O33" s="4" t="n">
         <v>0</v>
@@ -3688,22 +4223,37 @@
       <c r="T33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U33" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V33" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W33" s="4" t="inlineStr">
+      <c r="U33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB33" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X33" s="4" t="inlineStr">
+      <c r="AC33" s="4" t="inlineStr">
         <is>
           <t>Certification-first publishing route.</t>
         </is>
@@ -3762,11 +4312,11 @@
       <c r="L34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="4" t="n">
-        <v>0</v>
+      <c r="M34" s="4" t="inlineStr"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O34" s="4" t="n">
         <v>0</v>
@@ -3786,22 +4336,37 @@
       <c r="T34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U34" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V34" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W34" s="4" t="inlineStr">
+      <c r="U34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB34" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X34" s="4" t="inlineStr">
+      <c r="AC34" s="4" t="inlineStr">
         <is>
           <t>Managed STR/direct-booking inventory and potential distribution partner.</t>
         </is>
@@ -3860,11 +4425,11 @@
       <c r="L35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="4" t="n">
-        <v>0</v>
+      <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O35" s="4" t="n">
         <v>0</v>
@@ -3884,22 +4449,37 @@
       <c r="T35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U35" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W35" s="4" t="inlineStr">
+      <c r="U35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB35" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X35" s="4" t="inlineStr">
+      <c r="AC35" s="4" t="inlineStr">
         <is>
           <t>Geospatial backbone for building matching.</t>
         </is>
@@ -3958,11 +4538,11 @@
       <c r="L36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="4" t="n">
-        <v>0</v>
+      <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O36" s="4" t="n">
         <v>0</v>
@@ -3982,22 +4562,37 @@
       <c r="T36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U36" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V36" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W36" s="4" t="inlineStr">
+      <c r="U36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB36" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X36" s="4" t="inlineStr">
+      <c r="AC36" s="4" t="inlineStr">
         <is>
           <t>Black Sea property management and STR inventory.</t>
         </is>
@@ -4056,11 +4651,11 @@
       <c r="L37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="4" t="n">
-        <v>0</v>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O37" s="4" t="n">
         <v>0</v>
@@ -4080,22 +4675,37 @@
       <c r="T37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W37" s="4" t="inlineStr">
+      <c r="U37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB37" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X37" s="4" t="inlineStr">
+      <c r="AC37" s="4" t="inlineStr">
         <is>
           <t>Verification layer, not acquisition feed.</t>
         </is>
@@ -4154,11 +4764,11 @@
       <c r="L38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="M38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="4" t="n">
-        <v>0</v>
+      <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O38" s="4" t="n">
         <v>0</v>
@@ -4178,22 +4788,37 @@
       <c r="T38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U38" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V38" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W38" s="4" t="inlineStr">
+      <c r="U38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB38" s="4" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X38" s="4" t="inlineStr">
+      <c r="AC38" s="4" t="inlineStr">
         <is>
           <t>Not a crawl-first source.</t>
         </is>
@@ -4252,11 +4877,11 @@
       <c r="L39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="5" t="n">
-        <v>0</v>
+      <c r="M39" s="5" t="inlineStr"/>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O39" s="5" t="n">
         <v>0</v>
@@ -4276,22 +4901,37 @@
       <c r="T39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U39" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V39" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W39" s="5" t="inlineStr">
+      <c r="U39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB39" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X39" s="5" t="inlineStr">
+      <c r="AC39" s="5" t="inlineStr">
         <is>
           <t>Do not rely on unstable login-restricted scraping.</t>
         </is>
@@ -4350,11 +4990,11 @@
       <c r="L40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="5" t="n">
-        <v>0</v>
+      <c r="M40" s="5" t="inlineStr"/>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O40" s="5" t="n">
         <v>0</v>
@@ -4374,22 +5014,37 @@
       <c r="T40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U40" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V40" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W40" s="5" t="inlineStr">
+      <c r="U40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB40" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X40" s="5" t="inlineStr">
+      <c r="AC40" s="5" t="inlineStr">
         <is>
           <t>Treat as agency-branding and lead overlay.</t>
         </is>
@@ -4440,54 +5095,69 @@
         </is>
       </c>
       <c r="J41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="5" t="inlineStr"/>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="K41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="P41" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V41" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="R41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T41" s="5" t="n">
+      <c r="W41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="U41" s="5" t="inlineStr">
+      <c r="Z41" s="5" t="inlineStr">
         <is>
           <t>long_term_rent, sale</t>
         </is>
       </c>
-      <c r="V41" s="5" t="inlineStr">
+      <c r="AA41" s="5" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W41" s="5" t="inlineStr">
+      <c r="AB41" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X41" s="5" t="inlineStr">
+      <c r="AC41" s="5" t="inlineStr">
         <is>
           <t>Lead-intelligence overlay only.</t>
         </is>
@@ -4542,11 +5212,11 @@
       <c r="L42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" s="5" t="n">
-        <v>0</v>
+      <c r="M42" s="5" t="inlineStr"/>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O42" s="5" t="n">
         <v>0</v>
@@ -4566,22 +5236,37 @@
       <c r="T42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U42" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V42" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W42" s="5" t="inlineStr">
+      <c r="U42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB42" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X42" s="5" t="inlineStr">
+      <c r="AC42" s="5" t="inlineStr">
         <is>
           <t>Deferred overlay until official/public read coverage is confirmed.</t>
         </is>
@@ -4640,11 +5325,11 @@
       <c r="L43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" s="5" t="n">
-        <v>0</v>
+      <c r="M43" s="5" t="inlineStr"/>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O43" s="5" t="n">
         <v>0</v>
@@ -4664,22 +5349,37 @@
       <c r="T43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U43" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V43" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W43" s="5" t="inlineStr">
+      <c r="U43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB43" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X43" s="5" t="inlineStr">
+      <c r="AC43" s="5" t="inlineStr">
         <is>
           <t>Privacy-restricted and unstructured.</t>
         </is>
@@ -4738,11 +5438,11 @@
       <c r="L44" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M44" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" s="5" t="n">
-        <v>0</v>
+      <c r="M44" s="5" t="inlineStr"/>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O44" s="5" t="n">
         <v>0</v>
@@ -4762,22 +5462,37 @@
       <c r="T44" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U44" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V44" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W44" s="5" t="inlineStr">
+      <c r="U44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z44" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA44" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB44" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X44" s="5" t="inlineStr">
+      <c r="AC44" s="5" t="inlineStr">
         <is>
           <t>Useful for owned-business communication, not broad scraping.</t>
         </is>
@@ -4828,28 +5543,28 @@
         </is>
       </c>
       <c r="J45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="5" t="inlineStr"/>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O45" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="K45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" s="5" t="n">
-        <v>0</v>
-      </c>
       <c r="P45" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q45" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R45" s="5" t="n">
         <v>0</v>
@@ -4858,31 +5573,46 @@
         <v>0</v>
       </c>
       <c r="T45" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="U45" s="5" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="U45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z45" s="5" t="inlineStr">
         <is>
           <t>sale</t>
         </is>
       </c>
-      <c r="V45" s="5" t="inlineStr">
+      <c r="AA45" s="5" t="inlineStr">
         <is>
           <t>apartment</t>
         </is>
       </c>
-      <c r="W45" s="5" t="inlineStr">
+      <c r="AB45" s="5" t="inlineStr">
         <is>
           <t>Blocked / deferred</t>
         </is>
       </c>
-      <c r="X45" s="5" t="inlineStr">
+      <c r="AC45" s="5" t="inlineStr">
         <is>
           <t>Useful mostly for market chatter and backlinks.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X45"/>
+  <autoFilter ref="A1:AC45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4893,7 +5623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4908,7 +5638,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-08 15:57 UTC</t>
+          <t>2026-04-09 09:52 UTC</t>
         </is>
       </c>
     </row>
@@ -4979,80 +5709,110 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Total Discovery Fixtures</t>
+          <t>Total Live Listings Parsed</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Total Discovery URLs Extracted</t>
+          <t>Total Live URLs Discovered</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Total Blocked/Error Fixtures</t>
+          <t>Total Live Photos Downloaded</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11</v>
+        <v>4351</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Total Photos in Fixtures</t>
+          <t>Total Discovery Fixtures</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Fixtures with Geo</t>
+          <t>Total Discovery URLs Extracted</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Fixtures with Address</t>
+          <t>Total Blocked/Error Fixtures</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Fixtures with Price</t>
+          <t>Total Photos in Fixtures</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>Fixtures with Geo</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Fixtures with Address</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Fixtures with Price</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
           <t>Fixtures with Area</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B19" t="n">
         <v>20</v>
       </c>
     </row>

</xml_diff>